<commit_message>
Disqualify biomass for clean heat ITC/PTC
</commit_message>
<xml_diff>
--- a/InputData/indst/IFTQfS/Indst Fuels Qualifying for Support.xlsx
+++ b/InputData/indst/IFTQfS/Indst Fuels Qualifying for Support.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\indst\IFTQfS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\IFTQfS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A26E8FDA-825D-45E0-9A1C-D179A264BAE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6495CBB6-BB3C-4AAF-9DDF-221DA0A91E08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{CEBBDD15-8244-44C2-A2EB-EB506D69E415}"/>
+    <workbookView xWindow="-26910" yWindow="1440" windowWidth="25980" windowHeight="14640" xr2:uid="{CEBBDD15-8244-44C2-A2EB-EB506D69E415}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -623,7 +623,7 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +743,7 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -863,7 +863,7 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>